<commit_message>
Curva S actualizada 2026-07-18 10:30 Chile
</commit_message>
<xml_diff>
--- a/data/50001451 - ZITRON COLOMBIA.xlsx
+++ b/data/50001451 - ZITRON COLOMBIA.xlsx
@@ -4648,7 +4648,7 @@
         <v>46107.840353321764</v>
       </c>
       <c r="D48" s="5">
-        <v>46107.84042637731</v>
+        <v>46220.94303859954</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>167</v>
@@ -5352,7 +5352,7 @@
         <v>46114.767718206014</v>
       </c>
       <c r="D60" s="5">
-        <v>46114.84872589121</v>
+        <v>46221.07565987269</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>200</v>
@@ -5661,7 +5661,7 @@
         <v>46114.78855440972</v>
       </c>
       <c r="D65" s="8">
-        <v>46114.78855586806</v>
+        <v>46221.38854112268</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>222</v>
@@ -5714,7 +5714,7 @@
         <v>46114.78858121528</v>
       </c>
       <c r="D66" s="5">
-        <v>46114.7885828125</v>
+        <v>46221.38859300926</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>225</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-29 21:10 UTC
</commit_message>
<xml_diff>
--- a/data/50001451 - ZITRON COLOMBIA.xlsx
+++ b/data/50001451 - ZITRON COLOMBIA.xlsx
@@ -10711,7 +10711,7 @@
       </c>
       <c r="C155" s="9"/>
       <c r="D155" s="8">
-        <v>46114.650831747684</v>
+        <v>46232.710285810186</v>
       </c>
       <c r="E155" s="9" t="s">
         <v>428</v>
@@ -10756,9 +10756,11 @@
       <c r="B156" s="5">
         <v>46077.82017730324</v>
       </c>
-      <c r="C156" s="6"/>
+      <c r="C156" s="5">
+        <v>46232.710263773144</v>
+      </c>
       <c r="D156" s="5">
-        <v>46137.18802717593</v>
+        <v>46232.71026662037</v>
       </c>
       <c r="E156" s="6" t="s">
         <v>431</v>
@@ -10819,9 +10821,11 @@
       <c r="B157" s="8">
         <v>46077.82017756945</v>
       </c>
-      <c r="C157" s="9"/>
+      <c r="C157" s="8">
+        <v>46232.71028025463</v>
+      </c>
       <c r="D157" s="8">
-        <v>46137.18802714121</v>
+        <v>46232.71028196759</v>
       </c>
       <c r="E157" s="9" t="s">
         <v>436</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-08-03 13:45 UTC
</commit_message>
<xml_diff>
--- a/data/50001451 - ZITRON COLOMBIA.xlsx
+++ b/data/50001451 - ZITRON COLOMBIA.xlsx
@@ -8527,7 +8527,7 @@
         <v>46121.840045046294</v>
       </c>
       <c r="D115" s="8">
-        <v>46225.80624795139</v>
+        <v>46237.56487802083</v>
       </c>
       <c r="E115" s="9" t="s">
         <v>351</v>
@@ -8588,9 +8588,11 @@
       <c r="B116" s="5">
         <v>46107.6021821412</v>
       </c>
-      <c r="C116" s="6"/>
+      <c r="C116" s="5">
+        <v>46237.56487096065</v>
+      </c>
       <c r="D116" s="5">
-        <v>46225.80624259259</v>
+        <v>46237.56487265046</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>225</v>
@@ -9134,7 +9136,7 @@
         <v>46122.612434027775</v>
       </c>
       <c r="D126" s="5">
-        <v>46225.80624855324</v>
+        <v>46237.564880034726</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>225</v>

</xml_diff>